<commit_message>
feat(server): PB numbers reset monthly from 1 per PT (PB/<kode PT>/<YYMM>/0001)
Owner decision 2026-10-11: DEFAULT_SEQUENCES expense_request → monthly, startAt 1
(retires the never + 229 paper series). Data migration 20261012_300200_d1010_pb_monthly
moves only sequences on the default pattern (audited, customised ones logged) and seeds
each month that already has issued PB numbers of the new shape at max(seq)+1, so the
current month continues without duplicates; down restores never/229 for moved rows.
Import: nomor_pb_mulai = first number of the go-live month (default 1), never the
sequence startAt. No built-in PT code: PDF / import use companies.shortCode only.
Tests: two PTs with independent monthly series, migration up/down, numbering suite.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRGH83oyWQDQ7pEfHDPg1g
</commit_message>
<xml_diff>
--- a/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
+++ b/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
@@ -315,7 +315,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nomor urut Pengajuan Biaya (PB) pertama di sistem (Q-17: melanjutkan nomor manual, 229). Contoh hasil: 229/PB-DRMS/01/X/2026. Per PT bisa diganti di sheet Perusahaan (kolom nomor_pb_mulai).</t>
+          <t xml:space="preserve">Nomor urut Pengajuan Biaya (PB) pertama di BULAN go-live (nomor PB direset tiap bulan mulai 1). Contoh hasil: PB/&lt;kode PT&gt;/2611/0001. Isi lebih dari 1 hanya bila bulan go-live melanjutkan nomor manual. Per PT bisa diganti di sheet Perusahaan (kolom nomor_pb_mulai).</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nomor urut Pengajuan Biaya (PB) pertama di sistem (Q-17: melanjutkan nomor manual, 229). Contoh hasil: 229/PB-DRMS/01/X/2026. Per PT bisa diganti di sheet Perusahaan (kolom nomor_pb_mulai).</t>
+          <t xml:space="preserve">Nomor urut Pengajuan Biaya (PB) pertama di BULAN go-live (nomor PB direset tiap bulan mulai 1). Contoh hasil: PB/&lt;kode PT&gt;/2611/0001. Isi lebih dari 1 hanya bila bulan go-live melanjutkan nomor manual. Per PT bisa diganti di sheet Perusahaan (kolom nomor_pb_mulai).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(import): Site sheet and kode_site on Karyawan/Project/Penugasan/AkunKas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRGH83oyWQDQ7pEfHDPg1g
</commit_message>
<xml_diff>
--- a/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
+++ b/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
@@ -17,12 +17,13 @@
     <sheet name="AksesPT" sheetId="9" r:id="rId9"/>
     <sheet name="Rekening" sheetId="10" r:id="rId10"/>
     <sheet name="PusatBiaya" sheetId="11" r:id="rId11"/>
-    <sheet name="Project" sheetId="12" r:id="rId12"/>
-    <sheet name="Tahapan" sheetId="13" r:id="rId13"/>
-    <sheet name="RAB" sheetId="14" r:id="rId14"/>
-    <sheet name="Kendaraan" sheetId="15" r:id="rId15"/>
-    <sheet name="Penugasan" sheetId="16" r:id="rId16"/>
-    <sheet name="AkunKas" sheetId="17" r:id="rId17"/>
+    <sheet name="Site" sheetId="12" r:id="rId12"/>
+    <sheet name="Project" sheetId="13" r:id="rId13"/>
+    <sheet name="Tahapan" sheetId="14" r:id="rId14"/>
+    <sheet name="RAB" sheetId="15" r:id="rId15"/>
+    <sheet name="Kendaraan" sheetId="16" r:id="rId16"/>
+    <sheet name="Penugasan" sheetId="17" r:id="rId17"/>
+    <sheet name="AkunKas" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -140,7 +141,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Versi template MC2-5. SEMUA DATA DI FILE INI FIKTIF (untuk uji/latihan), bukan data klien.</t>
+          <t xml:space="preserve">Versi template MC2-5 + Site (ADR 0023). SEMUA DATA DI FILE INI FIKTIF (untuk uji/latihan), bukan data klien.</t>
         </is>
       </c>
     </row>
@@ -749,166 +750,161 @@
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional: site penempatan (sheet Site, PT yang sama) — boleh absen di site ini tanpa penugasan. Kosong = tidak diubah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pengguna</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pengguna (akun login) + peran: Orang yang login ke web/APK (satu baris per orang). Akun login (password) dibuat oleh Lead di Keycloak realm drms — di file ini TIDAK ADA password. peran + kode_karyawan = akses di PT kode_pt (Direktur, Finance, PM, Staff, Admin; boleh lebih dari satu, dipisah koma). Akses di PT lain: sheet AksesPT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pt</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">username</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama login: huruf kecil/angka/titik/minus, 3–64 karakter, unik. Mis. budi.h</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">username</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional (Q-37). Dipakai untuk reset password; kosong = reset oleh Admin.</t>
+          <t xml:space="preserve">Nama login: huruf kecil/angka/titik/minus, 3–64 karakter, unik. Mis. budi.h</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">nama</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama tampilan.</t>
+          <t xml:space="preserve">Opsional (Q-37). Dipakai untuk reset password; kosong = reset oleh Admin.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_karyawan</t>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode karyawan di PT kode_pt (sheet Karyawan). Wajib untuk Staff/PM yang mengajukan atau absen.</t>
+          <t xml:space="preserve">Nama tampilan.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">peran</t>
+          <t xml:space="preserve">kode_karyawan</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peran di PT kode_pt: Direktur, Finance, PM, Staff, Admin (pisahkan dengan koma). Kosong = tanpa akses di PT itu (isi sheet AksesPT).</t>
+          <t xml:space="preserve">Kode karyawan di PT kode_pt (sheet Karyawan). Wajib untuk Staff/PM yang mengajukan atau absen.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">no_hp</t>
+          <t xml:space="preserve">peran</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional.</t>
+          <t xml:space="preserve">Peran di PT kode_pt: Direktur, Finance, PM, Staff, Admin (pisahkan dengan koma). Kosong = tanpa akses di PT itu (isi sheet AksesPT).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
+          <t xml:space="preserve">no_hp</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="7" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">AksesPT</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Akses pengguna di PT lain: Opsional (MC2-5): peran pengguna di PT SELAIN kode_pt barisnya di sheet Pengguna — satu baris per pengguna per PT. Peran bisa berbeda per PT (mis. Direktur di DRMS, Finance di CS1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">username</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Username (sheet Pengguna).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pt</t>
+          <t xml:space="preserve">username</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -918,14 +914,14 @@
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada).</t>
+          <t xml:space="preserve">Username (sheet Pengguna).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">peran</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -935,79 +931,79 @@
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peran di PT ini: Direktur, Finance, PM, Staff, Admin (pisahkan dengan koma).</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_karyawan</t>
+          <t xml:space="preserve">peran</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional: kode karyawan di PT ini (sheet Karyawan, kode_pt sama).</t>
+          <t xml:space="preserve">Peran di PT ini: Direktur, Finance, PM, Staff, Admin (pisahkan dengan koma).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_karyawan</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional: kode karyawan di PT ini (sheet Karyawan, kode_pt sama).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="7" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Rekening</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Rekening karyawan: Rekening tujuan transfer pengajuan. Satu karyawan boleh punya beberapa rekening; tandai satu sebagai default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pt</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_karyawan</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode karyawan (sheet Karyawan).</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_bank</t>
+          <t xml:space="preserve">kode_karyawan</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1017,14 +1013,14 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode bank (sheet Bank).</t>
+          <t xml:space="preserve">Kode karyawan (sheet Karyawan).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">no_rekening</t>
+          <t xml:space="preserve">kode_bank</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1034,14 +1030,14 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hanya angka 5–34 digit (format teks agar nol di depan tidak hilang).</t>
+          <t xml:space="preserve">Kode bank (sheet Bank).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">atas_nama</t>
+          <t xml:space="preserve">no_rekening</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1051,79 +1047,79 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama pemilik rekening sesuai buku tabungan.</t>
+          <t xml:space="preserve">Hanya angka 5–34 digit (format teks agar nol di depan tidak hilang).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">rekening_default</t>
+          <t xml:space="preserve">atas_nama</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ya untuk rekening utama (maks. satu per karyawan).</t>
+          <t xml:space="preserve">Nama pemilik rekening sesuai buku tabungan.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
+          <t xml:space="preserve">rekening_default</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya untuk rekening utama (maks. satu per karyawan).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D78" s="5" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="7" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PusatBiaya</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pusat biaya / lokasi operasional: Lokasi operasional non-project (Q-23), mis. "Ops Palangka Banjar", dengan penanggung jawab dan koordinat absen (Q-40).</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pt</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode unik per PT, mis. OPS-PB.</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">nama</t>
+          <t xml:space="preserve">kode</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1133,127 +1129,127 @@
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama lokasi.</t>
+          <t xml:space="preserve">Kode unik per PT, mis. OPS-PB.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">jenis</t>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operasional atau Departemen. Kosong = Operasional.</t>
+          <t xml:space="preserve">Nama lokasi.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">penanggung_jawab</t>
+          <t xml:space="preserve">jenis</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Username penanggung jawab (sheet Pengguna).</t>
+          <t xml:space="preserve">Operasional atau Departemen. Kosong = Operasional.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">latitude</t>
+          <t xml:space="preserve">penanggung_jawab</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama).</t>
+          <t xml:space="preserve">Username penanggung jawab (sheet Pengguna).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">longitude</t>
+          <t xml:space="preserve">latitude</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps).</t>
+          <t xml:space="preserve">Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">radius_m</t>
+          <t xml:space="preserve">longitude</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi.</t>
+          <t xml:space="preserve">Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
+          <t xml:space="preserve">radius_m</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Project</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Project: Project konstruksi yang sedang berjalan saat go-live, dengan PM, koordinat lokasi (absen) dan RAB total.</t>
-        </is>
-      </c>
-    </row>
     <row r="90">
-      <c r="B90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pt</t>
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Site</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Site (kantor cabang): Kantor cabang PT (ADR 0023), mis. "Cabang Balikpapan": satu site menangani beberapa project. Koordinat = titik absen kantor cabang; pusat biaya default = pusat biaya operasional cabang. Dihubungkan lewat kolom kode_site di sheet Karyawan, Project, Penugasan dan AkunKas.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode project unik per PT, mis. PRJ-2026-01.</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">nama</t>
+          <t xml:space="preserve">kode</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1263,19 +1259,24 @@
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama project.</t>
+          <t xml:space="preserve">Kode site unik per PT, mis. CAB-BPN.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">klien</t>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional: nama klien/pemberi kerja (dibuat otomatis bila belum ada).</t>
+          <t xml:space="preserve">Nama site, mis. Cabang Balikpapan.</t>
         </is>
       </c>
     </row>
@@ -1294,311 +1295,281 @@
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">pm</t>
+          <t xml:space="preserve">latitude</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Username PM (sheet Pengguna).</t>
+          <t xml:space="preserve">Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">latitude</t>
+          <t xml:space="preserve">longitude</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama).</t>
+          <t xml:space="preserve">Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">longitude</t>
+          <t xml:space="preserve">radius_m</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps).</t>
+          <t xml:space="preserve">Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">radius_m</t>
+          <t xml:space="preserve">kode_pusat_biaya</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi.</t>
+          <t xml:space="preserve">Opsional: pusat biaya default (operasional, sheet PusatBiaya, PT yang sama).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">rab</t>
+          <t xml:space="preserve">aktif</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini.</t>
+          <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="B100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tanggal_mulai</t>
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Project</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Format YYYY-MM-DD atau DD/MM/YYYY.</t>
+          <t xml:space="preserve">Project: Project konstruksi yang sedang berjalan saat go-live, dengan PM, koordinat lokasi (absen) dan RAB total.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">target_selesai</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Format YYYY-MM-DD atau DD/MM/YYYY.</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">kode</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perencanaan, Berjalan, Ditunda, Selesai. Kosong = Berjalan.</t>
+          <t xml:space="preserve">Kode project unik per PT, mis. PRJ-2026-01.</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tahapan</t>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tahapan project + bobot: Tahapan pekerjaan per project. Total bobot tahapan satu project harus tepat 100%. Progress awal tahapan = 0% (diisi lewat laporan progress).</t>
+          <t xml:space="preserve">Nama project.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pt</t>
+          <t xml:space="preserve">klien</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Opsional: nama klien/pemberi kerja (dibuat otomatis bila belum ada).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_project</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">alamat</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode project (sheet Project).</t>
+          <t xml:space="preserve">Opsional.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">urutan</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">pm</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nomor urut tahapan 1, 2, 3, …</t>
+          <t xml:space="preserve">Username PM (sheet Pengguna).</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">nama</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_site</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama tahapan, mis. Pondasi.</t>
+          <t xml:space="preserve">Opsional: site (kantor cabang) yang menangani project ini (sheet Site, PT yang sama). Kosong = tidak diubah.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">bobot_persen</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">latitude</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bobot 0–100; jumlah per project = 100.</t>
+          <t xml:space="preserve">Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama).</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RAB</t>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">longitude</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAB per kategori: Opsional: anggaran project per kategori pengeluaran (untuk laporan realisasi vs RAB).</t>
+          <t xml:space="preserve">Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps).</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pt</t>
+          <t xml:space="preserve">radius_m</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_project</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">rab</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode project (sheet Project).</t>
+          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_kategori</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">tanggal_mulai</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode kategori (sheet Kategori).</t>
+          <t xml:space="preserve">Format YYYY-MM-DD atau DD/MM/YYYY.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">nominal</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">target_selesai</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rupiah, bilangan bulat.</t>
+          <t xml:space="preserve">Format YYYY-MM-DD atau DD/MM/YYYY.</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kendaraan</t>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kendaraan / unit: Kendaraan untuk baris BBM/Service Kendaraan (Q-22).</t>
+          <t xml:space="preserve">Perencanaan, Berjalan, Ditunda, Selesai. Kosong = Berjalan.</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="B115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pt</t>
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tahapan</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Tahapan project + bobot: Tahapan pekerjaan per project. Total bobot tahapan satu project harus tepat 100%. Progress awal tahapan = 0% (diisi lewat laporan progress).</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">no_polisi</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mis. DA 1234 XY (spasi boleh).</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">jenis</t>
+          <t xml:space="preserve">kode_project</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -1608,86 +1579,106 @@
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mis. Hilux, Tronton.</t>
+          <t xml:space="preserve">Kode project (sheet Project).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">merek_model</t>
+          <t xml:space="preserve">urutan</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional.</t>
+          <t xml:space="preserve">Nomor urut tahapan 1, 2, 3, …</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pusat_biaya</t>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional: pusat biaya default (sheet PusatBiaya).</t>
+          <t xml:space="preserve">Nama tahapan, mis. Pondasi.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_project</t>
+          <t xml:space="preserve">bobot_persen</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional: project default (sheet Project).</t>
+          <t xml:space="preserve">Bobot 0–100; jumlah per project = 100.</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="B121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">aktif</t>
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAB</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
+          <t xml:space="preserve">RAB per kategori: Opsional: anggaran project per kategori pengeluaran (untuk laporan realisasi vs RAB).</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Penugasan</t>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penugasan tim: Karyawan yang ditugaskan ke project ATAU pusat biaya (menentukan project yang terlihat di APK dan lokasi absen).</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pt</t>
+          <t xml:space="preserve">kode_project</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Kode project (sheet Project).</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_karyawan</t>
+          <t xml:space="preserve">kode_kategori</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -1697,200 +1688,388 @@
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode karyawan (sheet Karyawan).</t>
+          <t xml:space="preserve">Kode kategori (sheet Kategori).</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_project</t>
+          <t xml:space="preserve">nominal</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isi salah satu: kode project …</t>
+          <t xml:space="preserve">Rupiah, bilangan bulat.</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="B126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_pusat_biaya</t>
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kendaraan</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">… ATAU kode pusat biaya.</t>
+          <t xml:space="preserve">Kendaraan / unit: Kendaraan untuk baris BBM/Service Kendaraan (Q-22).</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">peran</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Staff, Mandor atau PM. Kosong = Staff.</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">tanggal_mulai</t>
+          <t xml:space="preserve">no_polisi</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional, YYYY-MM-DD atau DD/MM/YYYY.</t>
+          <t xml:space="preserve">Mis. DA 1234 XY (spasi boleh).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">tanggal_selesai</t>
+          <t xml:space="preserve">jenis</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Mis. Hilux, Tronton.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">merek_model</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Opsional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AkunKas</t>
-        </is>
-      </c>
-      <c r="D130" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Akun kas/bank perusahaan + saldo awal: Akun kas dan rekening bank perusahaan dengan saldo per tanggal go-live (sheet Pengaturan). Saldo awal dikunci setelah periode pertama sejak go-live ditutup.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_pt</t>
+          <t xml:space="preserve">kode_pusat_biaya</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+          <t xml:space="preserve">Opsional: pusat biaya default (sheet PusatBiaya).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">nama</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_project</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama akun unik per PT, mis. Kas Kecil, Bank Mandiri Operasional.</t>
+          <t xml:space="preserve">Opsional: project default (sheet Project).</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">jenis</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">aktif</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kas atau Bank.</t>
+          <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="B134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kode_bank</t>
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Penugasan</t>
         </is>
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Untuk jenis Bank: kode bank (sheet Bank).</t>
+          <t xml:space="preserve">Penugasan tim: Karyawan yang ditugaskan ke project, pusat biaya ATAU site (menentukan project yang terlihat di APK dan lokasi absen).</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">no_rekening</t>
+          <t xml:space="preserve">kode_pt</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Untuk jenis Bank: nomor rekening (teks).</t>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">atas_nama</t>
+          <t xml:space="preserve">kode_karyawan</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional.</t>
+          <t xml:space="preserve">Kode karyawan (sheet Karyawan).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">saldo_awal</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">kode_project</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saldo pada tanggal go-live (Rupiah, bilangan bulat ≥ 0).</t>
+          <t xml:space="preserve">Isi salah satu: kode project …</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">kode_jurnal_odoo</t>
+          <t xml:space="preserve">kode_pusat_biaya</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opsional.</t>
+          <t xml:space="preserve">… ATAU kode pusat biaya …</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">… ATAU kode site (kantor cabang, sheet Site).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">peran</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff, Mandor atau PM. Kosong = Staff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tanggal_mulai</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional, YYYY-MM-DD atau DD/MM/YYYY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tanggal_selesai</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AkunKas</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Akun kas/bank perusahaan + saldo awal: Akun kas dan rekening bank perusahaan dengan saldo per tanggal go-live (sheet Pengaturan). Saldo awal dikunci setelah periode pertama sejak go-live ditutup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_pt</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nama</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nama akun unik per PT, mis. Kas Kecil, Bank Mandiri Operasional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jenis</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kas atau Bank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_bank</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untuk jenis Bank: kode bank (sheet Bank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no_rekening</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untuk jenis Bank: nomor rekening (teks).</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">atas_nama</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">saldo_awal</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saldo pada tanggal go-live (Rupiah, bilangan bulat ≥ 0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_jurnal_odoo</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opsional: kas kecil / rekening site ini (sheet Site, PT yang sama). Kosong = tidak diubah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
-      <c r="D139" s="5" t="inlineStr">
+      <c r="D153" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya/Tidak. Kosong = Ya.</t>
         </is>
@@ -2296,18 +2475,153 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1" style="3"/>
+    <col min="2" max="2" width="12" customWidth="1" style="3"/>
+    <col min="3" max="3" width="26" customWidth="1" style="3"/>
+    <col min="4" max="4" width="28" customWidth="1" style="3"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1" style="3"/>
+    <col min="9" max="9" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_pt</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode *</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nama *</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alamat</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">latitude</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">longitude</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">radius_m</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kode_pusat_biaya</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aktif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DRMS</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-CAB</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cabang Contoh (FIKTIF)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jl. Cabang Contoh No. 3, Kota Fiktif</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>-2.2105</v>
+      </c>
+      <c r="F2">
+        <v>113.9208</v>
+      </c>
+      <c r="G2">
+        <v>120</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-OPS</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pt" prompt="Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT." sqref="A2:A2000">
+      <formula1>Perusahaan!$A$2:$A$2000</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="kode" prompt="Kode site unik per PT, mis. CAB-BPN." sqref="B2:B2000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="nama" prompt="Nama site, mis. Cabang Balikpapan." sqref="C2:C2000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="alamat" prompt="Opsional." sqref="D2:D2000"/>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -90 s.d. 90." showInputMessage="1" promptTitle="latitude" prompt="Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama)." sqref="E2:E2000">
+      <formula1>-90</formula1>
+      <formula2>90</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -180 s.d. 180." showInputMessage="1" promptTitle="longitude" prompt="Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps)." sqref="F2:F2000">
+      <formula1>-180</formula1>
+      <formula2>180</formula2>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat 10 s.d. 5000." showInputMessage="1" promptTitle="radius_m" prompt="Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi." sqref="G2:G2000">
+      <formula1>10</formula1>
+      <formula2>5000</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pusat_biaya" prompt="Opsional: pusat biaya default (operasional, sheet PusatBiaya, PT yang sama)." sqref="H2:H2000">
+      <formula1>PusatBiaya!$B$2:$B$2000</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="aktif" prompt="Ya/Tidak. Kosong = Ya." sqref="I2:I2000">
+      <formula1>"Ya,Tidak"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1" style="3"/>
     <col min="2" max="2" width="14" customWidth="1" style="3"/>
     <col min="3" max="3" width="30" customWidth="1" style="3"/>
     <col min="4" max="4" width="22" customWidth="1" style="3"/>
     <col min="5" max="5" width="28" customWidth="1" style="3"/>
     <col min="6" max="6" width="16" customWidth="1" style="3"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1" style="3"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1" style="3"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1" style="3"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1" style="3"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2343,35 +2657,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">latitude</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">longitude</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">radius_m</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">rab</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">tanggal_mulai</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">target_selesai</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">status</t>
         </is>
@@ -2408,26 +2727,26 @@
           <t xml:space="preserve">candra.contoh</t>
         </is>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>-3.3199</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>114.5901</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>200</v>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-08-01</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2027-03-31</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">Berjalan</t>
         </is>
@@ -2459,29 +2778,34 @@
           <t xml:space="preserve">candra.contoh</t>
         </is>
       </c>
-      <c r="G3">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-CAB</t>
+        </is>
+      </c>
+      <c r="H3">
         <v>-3.4402</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>114.8303</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>300</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>350000000</v>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2027-01-31</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">Berjalan</t>
         </is>
@@ -2508,31 +2832,31 @@
           <t xml:space="preserve">candra.contoh</t>
         </is>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>-3.3</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>114.6</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>150</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>20000000</v>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-11-01</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">Berjalan</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="14">
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pt" prompt="Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT." sqref="A2:A2000">
       <formula1>Perusahaan!$A$2:$A$2000</formula1>
     </dataValidation>
@@ -2543,24 +2867,27 @@
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="pm" prompt="Username PM (sheet Pengguna)." sqref="F2:F2000">
       <formula1>Pengguna!$B$2:$B$2000</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -90 s.d. 90." showInputMessage="1" promptTitle="latitude" prompt="Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama)." sqref="G2:G2000">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_site" prompt="Opsional: site (kantor cabang) yang menangani project ini (sheet Site, PT yang sama). Kosong = tidak diubah." sqref="G2:G2000">
+      <formula1>Site!$B$2:$B$2000</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -90 s.d. 90." showInputMessage="1" promptTitle="latitude" prompt="Derajat desimal, mis. -2.2136 (Google Maps: klik kanan lokasi → salin angka pertama)." sqref="H2:H2000">
       <formula1>-90</formula1>
       <formula2>90</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -180 s.d. 180." showInputMessage="1" promptTitle="longitude" prompt="Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps)." sqref="H2:H2000">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi angka -180 s.d. 180." showInputMessage="1" promptTitle="longitude" prompt="Derajat desimal, mis. 113.9108 (angka kedua dari Google Maps)." sqref="I2:I2000">
       <formula1>-180</formula1>
       <formula2>180</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat 10 s.d. 5000." showInputMessage="1" promptTitle="radius_m" prompt="Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi." sqref="I2:I2000">
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat 10 s.d. 5000." showInputMessage="1" promptTitle="radius_m" prompt="Radius absen (geofence) dalam meter, 10–5000. Wajib bila koordinat diisi." sqref="J2:J2000">
       <formula1>10</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini." sqref="J2:J2000">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini." sqref="K2:K2000">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="K2:K2000"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="target_selesai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="L2:L2000"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="status" prompt="Perencanaan, Berjalan, Ditunda, Selesai. Kosong = Berjalan." sqref="M2:M2000">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="L2:L2000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="target_selesai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="M2:M2000"/>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="status" prompt="Perencanaan, Berjalan, Ditunda, Selesai. Kosong = Berjalan." sqref="N2:N2000">
       <formula1>"Perencanaan,Berjalan,Ditunda,Selesai"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2568,7 +2895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2766,7 +3093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2897,7 +3224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3028,7 +3355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3036,9 +3363,10 @@
     <col min="2" max="2" width="14" customWidth="1" style="3"/>
     <col min="3" max="3" width="14" customWidth="1" style="3"/>
     <col min="4" max="4" width="16" customWidth="1" style="3"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1" style="3"/>
+    <col min="5" max="5" width="12" customWidth="1" style="3"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1" style="3"/>
+    <col min="8" max="8" width="13" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3064,15 +3392,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">peran</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">tanggal_mulai</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">tanggal_selesai</t>
         </is>
@@ -3094,12 +3427,12 @@
           <t xml:space="preserve">CTH-PRJ-01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-11-01</t>
         </is>
@@ -3121,12 +3454,12 @@
           <t xml:space="preserve">CTH-PRJ-01</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mandor</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-11-01</t>
         </is>
@@ -3148,7 +3481,7 @@
           <t xml:space="preserve">CTH-OPS</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff</t>
         </is>
@@ -3157,27 +3490,54 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">DRMS</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-005</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-CAB</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandor</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-11-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">CS1</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">CS1-001</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">CS1-GDG</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pt" prompt="Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT." sqref="A2:A2000">
       <formula1>Perusahaan!$A$2:$A$2000</formula1>
     </dataValidation>
@@ -3187,20 +3547,23 @@
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_project" prompt="Isi salah satu: kode project …" sqref="C2:C2000">
       <formula1>Project!$B$2:$B$2000</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pusat_biaya" prompt="… ATAU kode pusat biaya." sqref="D2:D2000">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pusat_biaya" prompt="… ATAU kode pusat biaya …" sqref="D2:D2000">
       <formula1>PusatBiaya!$B$2:$B$2000</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="peran" prompt="Staff, Mandor atau PM. Kosong = Staff." sqref="E2:E2000">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_site" prompt="… ATAU kode site (kantor cabang, sheet Site)." sqref="E2:E2000">
+      <formula1>Site!$B$2:$B$2000</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="peran" prompt="Staff, Mandor atau PM. Kosong = Staff." sqref="F2:F2000">
       <formula1>"Staff,Mandor,PM"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Opsional, YYYY-MM-DD atau DD/MM/YYYY." sqref="F2:F2000"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_selesai" prompt="Opsional." sqref="G2:G2000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Opsional, YYYY-MM-DD atau DD/MM/YYYY." sqref="G2:G2000"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_selesai" prompt="Opsional." sqref="H2:H2000"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3212,7 +3575,8 @@
     <col min="6" max="6" width="24" customWidth="1" style="3"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1" style="3"/>
-    <col min="9" max="9" width="9" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1" style="3"/>
+    <col min="10" max="10" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3258,6 +3622,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
@@ -3281,7 +3650,12 @@
       <c r="G2">
         <v>5000000</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-CAB</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -3326,7 +3700,7 @@
           <t xml:space="preserve">BNK1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -3351,14 +3725,14 @@
       <c r="G4">
         <v>1000000</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pt" prompt="Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT." sqref="A2:A2000">
       <formula1>Perusahaan!$A$2:$A$2000</formula1>
     </dataValidation>
@@ -3375,7 +3749,10 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="kode_jurnal_odoo" prompt="Opsional." sqref="H2:H2000"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="aktif" prompt="Ya/Tidak. Kosong = Ya." sqref="I2:I2000">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_site" prompt="Opsional: kas kecil / rekening site ini (sheet Site, PT yang sama). Kosong = tidak diubah." sqref="I2:I2000">
+      <formula1>Site!$B$2:$B$2000</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="aktif" prompt="Ya/Tidak. Kosong = Ya." sqref="J2:J2000">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4298,7 +4675,8 @@
     <col min="4" max="4" width="14" customWidth="1" style="3"/>
     <col min="5" max="5" width="18" customWidth="1" style="3"/>
     <col min="6" max="6" width="16" customWidth="1" style="3"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1" style="3"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4334,6 +4712,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">kode_site</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">aktif</t>
         </is>
       </c>
@@ -4369,7 +4752,7 @@
           <t xml:space="preserve">081200000001</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4406,7 +4789,7 @@
           <t xml:space="preserve">081200000002</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4443,7 +4826,7 @@
           <t xml:space="preserve">081200000003</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4480,7 +4863,7 @@
           <t xml:space="preserve">081200000004</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4512,7 +4895,7 @@
           <t xml:space="preserve">Mandor</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4544,7 +4927,12 @@
           <t xml:space="preserve">Admin</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CTH-CAB</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4581,7 +4969,7 @@
           <t xml:space="preserve">081200000003</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -4613,14 +5001,14 @@
           <t xml:space="preserve">Staff lapangan</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_pt" prompt="Kode PT (sheet Perusahaan atau PT yang sudah ada), mis. DRMS. Kosong = satu-satunya PT; wajib bila ada lebih dari satu PT." sqref="A2:A2000">
       <formula1>Perusahaan!$A$2:$A$2000</formula1>
     </dataValidation>
@@ -4629,7 +5017,10 @@
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="nama_panggilan" prompt="Opsional." sqref="D2:D2000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="jabatan" prompt="Opsional, mis. Mandor, Driver." sqref="E2:E2000"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="no_hp" prompt="Opsional, mis. 0812xxxx (format teks)." sqref="F2:F2000"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="aktif" prompt="Ya/Tidak. Kosong = Ya." sqref="G2:G2000">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="kode_site" prompt="Opsional: site penempatan (sheet Site, PT yang sama) — boleh absen di site ini tanpa penugasan. Kosong = tidak diubah." sqref="G2:G2000">
+      <formula1>Site!$B$2:$B$2000</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak ada di daftar" error="Pilih nilai dari daftar (lihat sheet Petunjuk)." showInputMessage="1" promptTitle="aktif" prompt="Ya/Tidak. Kosong = Ya." sqref="H2:H2000">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(server): D4 — RAP required for every project with a RAB (owner 2026-10-11)
Submit refused with 400 projectId "Project belum punya RAP — hubungi PM" for any kind with
RAB > 0 (konstruksi unchanged). RAP editor/import/templates for every kind: stage optional
outside konstruksi (DB guard), progress refresh konstruksi-only, templates per project kind.
API: rapRequired/rapMissing on projects, rapRequired/drivesProgress on /rap, nullable stage.
Migrations 20261013_400000/400100_d1010_rap_all (log of RAB projects without RAP).
Go-live import warns per project with RAB but no RAP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRGH83oyWQDQ7pEfHDPg1g
</commit_message>
<xml_diff>
--- a/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
+++ b/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
@@ -1347,7 +1347,7 @@
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini.</t>
+          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini. Project ber-RAB wajib punya RAP sebelum pengajuan dikirim: isi RAP setelah impor (tab RAP project).</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       <formula1>10</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini." sqref="J2:J2000">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini. Project ber-RAB wajib punya RAP sebelum pengajuan dikirim: isi RAP setelah impor (tab RAP project)." sqref="J2:J2000">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="K2:K2000"/>

</xml_diff>

<commit_message>
chore: regenerate importMap, OpenAPI, import templates and the latest migration snapshot after merging Phase D/E/F/G
The latest migration snapshot (20261013_400000_d1010_rap_all.json) now carries the loans, sites and
approval-config tables, so migrate:create reports no changes on the merged schema.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRGH83oyWQDQ7pEfHDPg1g
</commit_message>
<xml_diff>
--- a/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
+++ b/docs/proyekkas/templates/drms-impor-golive-contoh-fiktif-2pt.xlsx
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini.</t>
+          <t xml:space="preserve">RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini. Project ber-RAB wajib punya RAP sebelum pengajuan dikirim: isi RAP setelah impor (tab RAP project).</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       <formula1>10</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini." sqref="K2:K2000">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Isi bilangan bulat minimal 0." showInputMessage="1" promptTitle="rab" prompt="RAB total (Rupiah, bilangan bulat). Kosong = jumlah sheet RAB project ini. Project ber-RAB wajib punya RAP sebelum pengajuan dikirim: isi RAP setelah impor (tab RAP project)." sqref="K2:K2000">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="tanggal_mulai" prompt="Format YYYY-MM-DD atau DD/MM/YYYY." sqref="L2:L2000"/>

</xml_diff>